<commit_message>
Remove Petitfee from Ozon plan (per owner); keep Celimax + Round Lab + Santa
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
+++ b/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="План Озон октябрь — всё" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="План Озон октябрь" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -63,12 +63,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,11 +117,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -507,14 +507,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OZON — единый план: косметика (октябрь) + Деды Морозы (сезон Q4)</t>
+          <t>OZON — единый план: косметика (Celimax, Round Lab) + Деды Морозы (сезон Q4)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Косметика — месячный план. Санта — сезон окт–дек (столбец «октябрь» ≈ 25% сезона, ramp). Маржа реальная/оценка.</t>
+          <t>Косметика — месячный план. Санта — сезон окт–дек (столбец «октябрь» ≈ 25% сезона). Маржа реальная/оценка.</t>
         </is>
       </c>
     </row>
@@ -905,90 +905,78 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Итого Celimax</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="11" t="n">
+        <v>4257</v>
+      </c>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="11" t="n">
+        <v>1863654</v>
+      </c>
+      <c r="H17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>КОСМЕТИКА · ROUND LAB</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ROUND LAB 1025 DOKDO CLEANSER_150ml - </t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>5499</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>599</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>779</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>779</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>291</v>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>226689</v>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>держать/растить</t>
-        </is>
-      </c>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB 1025 DOKDO TONER_200ml / Отш</t>
+          <t xml:space="preserve">ROUND LAB 1025 DOKDO CLEANSER_150ml - </t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>802</v>
+        <v>5499</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>81</v>
+        <v>599</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0</v>
+        <v>779</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0</v>
+        <v>779</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>-419</v>
+        <v>291</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>минус — резать</t>
+        <v>226689</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>держать/растить</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB BIRCH JUICE MOISTURIZING CRE</t>
+          <t>ROUND LAB 1025 DOKDO TONER_200ml / Отш</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>102</v>
+        <v>802</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>5</v>
+        <v>81</v>
       </c>
       <c r="D20" s="6" t="n">
         <v>0</v>
@@ -997,7 +985,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>-543</v>
+        <v>-419</v>
       </c>
       <c r="G20" s="6" t="n">
         <v>0</v>
@@ -1011,1151 +999,645 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB MUGWORT CALMING CLEANSER_150</t>
+          <t>ROUND LAB BIRCH JUICE MOISTURIZING CRE</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>1201</v>
+        <v>102</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>290</v>
+        <v>-543</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>34800</v>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>0</v>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>минус — резать</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB PINE CALMING CICA AMPOULE_30</t>
+          <t>ROUND LAB MUGWORT CALMING CLEANSER_150</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>5</v>
+        <v>1201</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5</v>
+        <v>120</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>5</v>
+        <v>120</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>290</v>
       </c>
       <c r="G22" s="6" t="n">
+        <v>34800</v>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>ЗАПУСК</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ROUND LAB PINE CALMING CICA AMPOULE_30</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>290</v>
+      </c>
+      <c r="G23" s="6" t="n">
         <v>1450</v>
       </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>КОСМЕТИКА · PETITFEE</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
-    </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>PETITFEE - Pink Vita Brightening Eye P</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n">
-        <v>202</v>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>581</v>
-      </c>
-      <c r="G24" s="6" t="n">
-        <v>581</v>
-      </c>
-      <c r="H24" s="7" t="inlineStr">
-        <is>
-          <t>держать/растить</t>
-        </is>
-      </c>
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Итого Round Lab</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="11" t="n">
+        <v>904</v>
+      </c>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="11" t="n">
+        <v>262939</v>
+      </c>
+      <c r="H24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>PETITFEE - Cacao Energizing Hydrogel E</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>144</v>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>626</v>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>626</v>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>держать/растить</t>
-        </is>
-      </c>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>ДЕДЫ МОРОЗЫ · сезон Q4 (Озон)</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Aura Quartz Hydrogel Eye Pa</t>
+          <t>№3 с мишкой</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>89</v>
+        <v>10885</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>1</v>
+        <v>803</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>1606</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1</v>
+        <v>402</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>626</v>
+        <v>289</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>626</v>
-      </c>
-      <c r="H26" s="7" t="inlineStr">
-        <is>
-          <t>держать/растить</t>
+        <v>464134</v>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Agave Cooling Hydrogel Face</t>
+          <t>№11 в клетку</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>741</v>
+        <v>7385</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>0</v>
+        <v>1656</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>120</v>
+        <v>3312</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>120</v>
+        <v>828</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>400</v>
+        <v>198</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>655776</v>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>держать</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Collagen &amp; CoQ10 Hydrogel E</t>
+          <t>№5 с подарком</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>641</v>
+        <v>7463</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>0</v>
+        <v>434</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>120</v>
+        <v>868</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>120</v>
+        <v>217</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>400</v>
+        <v>231</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>200508</v>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Gold &amp; Snail Hydrogel Eye P</t>
+          <t>№6 блестящий</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>608</v>
+        <v>1519</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>0</v>
+        <v>510</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>120</v>
+        <v>1020</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>120</v>
+        <v>255</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>400</v>
+        <v>209</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>213180</v>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>держать</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Black Pearl &amp; Gold Hydrogel</t>
+          <t>№9 рябь</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>549</v>
+        <v>1290</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>0</v>
+        <v>296</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>120</v>
+        <v>592</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>400</v>
+        <v>238</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>140896</v>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Gold Hydrogel Mask Pack [5p</t>
+          <t>№1 красный</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>529</v>
+        <v>2579</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>120</v>
+        <v>720</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>400</v>
+        <v>224</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>161280</v>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PETITFEE - Agave Cooling Hydrogel Eye </t>
+          <t>№12 лыжи белые</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>0</v>
+        <v>310</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>120</v>
+        <v>620</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>400</v>
+        <v>210</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>130200</v>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>держать</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Bera Glucan Deep Firming Ey</t>
+          <t>№10 серый</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>406</v>
+        <v>2374</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>0</v>
+        <v>331</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>120</v>
+        <v>662</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>120</v>
+        <v>166</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>400</v>
+        <v>166</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>109892</v>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>держать</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Gold Hydrogel Eye Patch [60</t>
+          <t>№13 лыжи чёрн.</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>405</v>
+        <v>996</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>0</v>
+        <v>209</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>120</v>
+        <v>418</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>400</v>
+        <v>55</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>0</v>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>не грузить (минус)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Cacao Energizing Hydrogel M</t>
+          <t>СГ-Белая</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>399</v>
+        <v>1497</v>
       </c>
       <c r="C35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>400</v>
+        <v>180</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H35" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>72000</v>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Artichoke Soothing Hydrogel</t>
+          <t>СГ-Красная</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>327</v>
+        <v>722</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>400</v>
+        <v>180</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H36" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>72000</v>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Black Pearl &amp; Gold Hydrogel</t>
+          <t>№2 (нов)</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>292</v>
+        <v>990</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>400</v>
+        <v>180</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H37" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>72000</v>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PETITFEE - Gold &amp; Snail Hydrogel Mask </t>
+          <t>№7 (нов)</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>273</v>
+        <v>930</v>
       </c>
       <c r="C38" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>400</v>
+        <v>180</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H38" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>72000</v>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - Artichoke Soothing Hydrogel</t>
+          <t>№8 (нов)</t>
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>156</v>
+        <v>576</v>
       </c>
       <c r="C39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>400</v>
+        <v>180</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="H39" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>72000</v>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>PETITFEE - MASK 6 (блек, агава, какао,</t>
+          <t>№15 (нов)</t>
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>106</v>
+        <v>210</v>
       </c>
       <c r="C40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>106</v>
+        <v>210</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>106</v>
+        <v>52</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>400</v>
+        <v>180</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>42400</v>
-      </c>
-      <c r="H40" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
+        <v>37800</v>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>разгонять</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>PETITFEE - MASK 5 (блек, агава, какао,</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="C41" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="E41" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F41" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="G41" s="6" t="n">
-        <v>40000</v>
-      </c>
-      <c r="H41" s="9" t="inlineStr">
-        <is>
-          <t>ЗАПУСК</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>ДЕДЫ МОРОЗЫ · сезон Q4 (Озон)</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="n"/>
-      <c r="C42" s="11" t="n"/>
-      <c r="D42" s="11" t="n"/>
-      <c r="E42" s="11" t="n"/>
-      <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
-      <c r="H42" s="11" t="n"/>
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Итого Деды Морозы (сезон)</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="11" t="n">
+        <v>12028</v>
+      </c>
+      <c r="E41" s="11" t="n">
+        <v>3007</v>
+      </c>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="11" t="n">
+        <v>2473666</v>
+      </c>
+      <c r="H41" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>№3 с мишкой</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n">
-        <v>10885</v>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>803</v>
-      </c>
-      <c r="D43" s="6" t="n">
-        <v>1606</v>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>402</v>
-      </c>
-      <c r="F43" s="6" t="n">
-        <v>289</v>
-      </c>
-      <c r="G43" s="6" t="n">
-        <v>464134</v>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>ИТОГО ОКТЯБРЬ (косметика + ramp Санты): 2 745 010 ₽  8 168 шт</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>№11 в клетку</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="n">
-        <v>7385</v>
-      </c>
-      <c r="C44" s="6" t="n">
-        <v>1656</v>
-      </c>
-      <c r="D44" s="6" t="n">
-        <v>3312</v>
-      </c>
-      <c r="E44" s="6" t="n">
-        <v>828</v>
-      </c>
-      <c r="F44" s="6" t="n">
-        <v>198</v>
-      </c>
-      <c r="G44" s="6" t="n">
-        <v>655776</v>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>держать</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>№5 с подарком</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="n">
-        <v>7463</v>
-      </c>
-      <c r="C45" s="6" t="n">
-        <v>434</v>
-      </c>
-      <c r="D45" s="6" t="n">
-        <v>868</v>
-      </c>
-      <c r="E45" s="6" t="n">
-        <v>217</v>
-      </c>
-      <c r="F45" s="6" t="n">
-        <v>231</v>
-      </c>
-      <c r="G45" s="6" t="n">
-        <v>200508</v>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>СПРАВОЧНО — полный Q4: 4 600 259 ₽</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>№6 блестящий</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="n">
-        <v>1519</v>
-      </c>
-      <c r="C46" s="6" t="n">
-        <v>510</v>
-      </c>
-      <c r="D46" s="6" t="n">
-        <v>1020</v>
-      </c>
-      <c r="E46" s="6" t="n">
-        <v>255</v>
-      </c>
-      <c r="F46" s="6" t="n">
-        <v>209</v>
-      </c>
-      <c r="G46" s="6" t="n">
-        <v>213180</v>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>держать</t>
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Petitfee убран из плана (на Озоне почти не продавался).</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>№9 рябь</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="n">
-        <v>1290</v>
-      </c>
-      <c r="C47" s="6" t="n">
-        <v>296</v>
-      </c>
-      <c r="D47" s="6" t="n">
-        <v>592</v>
-      </c>
-      <c r="E47" s="6" t="n">
-        <v>148</v>
-      </c>
-      <c r="F47" s="6" t="n">
-        <v>238</v>
-      </c>
-      <c r="G47" s="6" t="n">
-        <v>140896</v>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>ВАЖНО: остаток Санты (43 тыс.) общий с WB — прогноз на Озон не складывать с WB-планом.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>№1 красный</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="n">
-        <v>2579</v>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>360</v>
-      </c>
-      <c r="D48" s="6" t="n">
-        <v>720</v>
-      </c>
-      <c r="E48" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="F48" s="6" t="n">
-        <v>224</v>
-      </c>
-      <c r="G48" s="6" t="n">
-        <v>161280</v>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>На FBO грузим только прогноз Санты, не весь остаток (72% не продастся за сезон).</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>№12 лыжи белые</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="n">
-        <v>3904</v>
-      </c>
-      <c r="C49" s="6" t="n">
-        <v>310</v>
-      </c>
-      <c r="D49" s="6" t="n">
-        <v>620</v>
-      </c>
-      <c r="E49" s="6" t="n">
-        <v>155</v>
-      </c>
-      <c r="F49" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="G49" s="6" t="n">
-        <v>130200</v>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>держать</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>№10 серый</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="n">
-        <v>2374</v>
-      </c>
-      <c r="C50" s="6" t="n">
-        <v>331</v>
-      </c>
-      <c r="D50" s="6" t="n">
-        <v>662</v>
-      </c>
-      <c r="E50" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="F50" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="G50" s="6" t="n">
-        <v>109892</v>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>держать</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>№13 лыжи чёрн.</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="n">
-        <v>996</v>
-      </c>
-      <c r="C51" s="6" t="n">
-        <v>209</v>
-      </c>
-      <c r="D51" s="6" t="n">
-        <v>418</v>
-      </c>
-      <c r="E51" s="6" t="n">
-        <v>104</v>
-      </c>
-      <c r="F51" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="G51" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="12" t="inlineStr">
-        <is>
-          <t>не грузить (минус)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>СГ-Белая</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="n">
-        <v>1497</v>
-      </c>
-      <c r="C52" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="E52" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F52" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="G52" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="H52" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>СГ-Красная</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="n">
-        <v>722</v>
-      </c>
-      <c r="C53" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="E53" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F53" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="G53" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="H53" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>№2 (нов)</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="n">
-        <v>990</v>
-      </c>
-      <c r="C54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="E54" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>№7 (нов)</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="n">
-        <v>930</v>
-      </c>
-      <c r="C55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="E55" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F55" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>№8 (нов)</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="n">
-        <v>576</v>
-      </c>
-      <c r="C56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="E56" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F56" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="G56" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="H56" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>№15 (нов)</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="C57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="F57" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="G57" s="6" t="n">
-        <v>37800</v>
-      </c>
-      <c r="H57" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>Итого Деды Морозы (сезон)</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="n"/>
-      <c r="C58" s="5" t="n"/>
-      <c r="D58" s="14" t="n">
-        <v>12028</v>
-      </c>
-      <c r="E58" s="14" t="n">
-        <v>3007</v>
-      </c>
-      <c r="F58" s="5" t="n"/>
-      <c r="G58" s="14" t="n">
-        <v>2473666</v>
-      </c>
-      <c r="H58" s="5" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="15" t="inlineStr">
-        <is>
-          <t>ИТОГО ОКТЯБРЬ (косметика + ramp Санты): 3 453 243 ₽ прибыли  9 937 шт</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="15" t="inlineStr">
-        <is>
-          <t>СПРАВОЧНО — полный Q4 (косметика×1 мес + весь сезон Санты): 5 308 492 ₽</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>Санта — сезонный товар (пик ноя–дек), поэтому показан сезон целиком + столбец «октябрь» (ramp ~25%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="16" t="inlineStr">
-        <is>
-          <t>ВАЖНО: остаток Санты (43 тыс.) общий с WB. Сезонный прогноз (~12 тыс. на Озон) НЕ складывать с WB-планом — товар один, делится между каналами.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="16" t="inlineStr">
-        <is>
-          <t>На FBO Озон грузим только прогноз Санты, не весь остаток — чтобы не платить хранение и вывоз (72% остатка не продастся за сезон).</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="16" t="inlineStr">
-        <is>
-          <t>Прибыль — цель при исполнении (реклама ≤15% ДРР, запуск показов Petitfee/Retinal, раскладка по кластерам). Реалистичный пол по косметике ~0,9–1,1 млн.</t>
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>Итоги — цель при исполнении (реклама ≤15% ДРР, запуск показов Retinal, раскладка по кластерам). Реалистичный пол по косметике ~0,9–1,1 млн.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A65:H65"/>
-    <mergeCell ref="A63:H63"/>
-    <mergeCell ref="A64:H64"/>
-    <mergeCell ref="A60:H60"/>
-    <mergeCell ref="A66:H66"/>
-    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A46:H46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add competitor columns to plan: LIFECOSM (Celimax), Cream.Shop (Round Lab)
Celimax rows show LIFECOSM per-product units/mo; Round Lab rows show
Cream.Shop's Round Lab category sales (RUB/mo, ~73% of Round Lab cleanser
market). Benchmarks make targets competitor-anchored.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
+++ b/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
@@ -491,30 +491,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OZON — единый план: косметика (Celimax, Round Lab) + Деды Морозы (сезон Q4)</t>
+          <t>OZON — план: косметика (Celimax, Round Lab) + Деды Морозы, с конкурентами</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Косметика — месячный план. Санта — сезон окт–дек (столбец «октябрь» ≈ 25% сезона). Маржа реальная/оценка.</t>
+          <t>Конкурент: Celimax → LIFECOSM (шт/мес, по товару); Round Lab → Cream.Shop (₽/мес по категории, ~73% рынка Round Lab).</t>
         </is>
       </c>
     </row>
@@ -531,30 +532,35 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Факт/пр. сезон</t>
+          <t>Факт/пр.сезон</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>План (окт/сезон), шт</t>
+          <t>Конкурент (прод.)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>в т.ч. октябрь</t>
+          <t>План, шт</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>в т.ч. окт</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Маржа/шт</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Прибыль (план)</t>
-        </is>
-      </c>
       <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Прибыль</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
@@ -573,11 +579,12 @@
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Celimax Dual Barrier Creamy Toner, тон</t>
+          <t>Celimax Dual Barrier Creamy Toner, т</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -586,19 +593,24 @@
       <c r="C6" s="6" t="n">
         <v>840</v>
       </c>
-      <c r="D6" s="6" t="n">
-        <v>1723</v>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 4354 шт</t>
+        </is>
       </c>
       <c r="E6" s="6" t="n">
         <v>1723</v>
       </c>
       <c r="F6" s="6" t="n">
+        <v>1723</v>
+      </c>
+      <c r="G6" s="6" t="n">
         <v>502</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="H6" s="6" t="n">
         <v>864946</v>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>растить к LIFECOSM</t>
         </is>
@@ -607,7 +619,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX THE VITA-A RETINOL SHOT TIGHTE</t>
+          <t>CELIMAX THE VITA-A RETINOL SHOT TIGH</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
@@ -616,19 +628,24 @@
       <c r="C7" s="6" t="n">
         <v>222</v>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>1336</v>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 4295 шт</t>
+        </is>
       </c>
       <c r="E7" s="6" t="n">
         <v>1336</v>
       </c>
       <c r="F7" s="6" t="n">
+        <v>1336</v>
+      </c>
+      <c r="G7" s="6" t="n">
         <v>442</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="H7" s="6" t="n">
         <v>590512</v>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>растить к LIFECOSM</t>
         </is>
@@ -637,7 +654,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX DUAL BARRIER SKIN WEARABLE CRE</t>
+          <t>CELIMAX DUAL BARRIER SKIN WEARABLE C</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -646,19 +663,24 @@
       <c r="C8" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="D8" s="6" t="n">
-        <v>0</v>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 1423 шт</t>
+        </is>
       </c>
       <c r="E8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6" t="n">
         <v>-52</v>
       </c>
-      <c r="G8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>минус — резать</t>
         </is>
@@ -667,7 +689,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX THE VITA-A RETINAL SHOT TIGHTE</t>
+          <t>CELIMAX THE VITA-A RETINAL SHOT TIGH</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -676,19 +698,24 @@
       <c r="C9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="6" t="n">
-        <v>684</v>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 4560 шт</t>
+        </is>
       </c>
       <c r="E9" s="6" t="n">
         <v>684</v>
       </c>
       <c r="F9" s="6" t="n">
+        <v>684</v>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="H9" s="6" t="n">
         <v>307800</v>
       </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
@@ -697,7 +724,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX PORE+DARK SPOT BRIGHTENING CRE</t>
+          <t>CELIMAX PORE+DARK SPOT BRIGHTENING C</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -706,19 +733,24 @@
       <c r="C10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="6" t="n">
-        <v>0</v>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="E10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>-637</v>
       </c>
-      <c r="G10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>минус — резать</t>
         </is>
@@ -727,7 +759,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX JI WOO GAE CICA BHA BLEMISH TO</t>
+          <t xml:space="preserve">CELIMAX JI WOO GAE CICA BHA BLEMISH </t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
@@ -736,19 +768,24 @@
       <c r="C11" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="6" t="n">
-        <v>0</v>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 850 шт</t>
+        </is>
       </c>
       <c r="E11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>-723</v>
       </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>минус — резать</t>
         </is>
@@ -757,7 +794,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX JI WOO GAE CICA BHA BLEMISH TO</t>
+          <t xml:space="preserve">CELIMAX JI WOO GAE CICA BHA BLEMISH </t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
@@ -766,19 +803,24 @@
       <c r="C12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="6" t="n">
-        <v>239</v>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 850 шт</t>
+        </is>
       </c>
       <c r="E12" s="6" t="n">
         <v>239</v>
       </c>
       <c r="F12" s="6" t="n">
+        <v>239</v>
+      </c>
+      <c r="G12" s="6" t="n">
         <v>164</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="H12" s="6" t="n">
         <v>39196</v>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>растить к LIFECOSM</t>
         </is>
@@ -787,7 +829,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX PORE+DARK SPOT BRIGHTENING PAD</t>
+          <t>CELIMAX PORE+DARK SPOT BRIGHTENING P</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
@@ -796,19 +838,24 @@
       <c r="C13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="6" t="n">
-        <v>139</v>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 928 шт</t>
+        </is>
       </c>
       <c r="E13" s="6" t="n">
         <v>139</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
@@ -817,7 +864,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX PORE+DARK SPOT BRIGHTENING SER</t>
+          <t>CELIMAX PORE+DARK SPOT BRIGHTENING S</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
@@ -826,19 +873,24 @@
       <c r="C14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="6" t="n">
-        <v>77</v>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 1080 шт</t>
+        </is>
       </c>
       <c r="E14" s="6" t="n">
         <v>77</v>
       </c>
       <c r="F14" s="6" t="n">
+        <v>77</v>
+      </c>
+      <c r="G14" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="H14" s="6" t="n">
         <v>34650</v>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
@@ -847,7 +899,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX THE REAL NONI ENERGY AMPOULE_3</t>
+          <t>CELIMAX THE REAL NONI ENERGY AMPOULE</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
@@ -856,19 +908,24 @@
       <c r="C15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>35</v>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 584 шт</t>
+        </is>
       </c>
       <c r="E15" s="6" t="n">
         <v>35</v>
       </c>
       <c r="F15" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G15" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="H15" s="6" t="n">
         <v>15750</v>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="I15" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
@@ -877,7 +934,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>CELIMAX THE REAL NONI MOISTURE BALANCI</t>
+          <t>CELIMAX THE REAL NONI MOISTURE BALAN</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
@@ -886,19 +943,24 @@
       <c r="C16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="6" t="n">
-        <v>24</v>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>LIFECOSM 1399 шт</t>
+        </is>
       </c>
       <c r="E16" s="6" t="n">
         <v>24</v>
       </c>
       <c r="F16" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G16" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="H16" s="6" t="n">
         <v>10800</v>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
@@ -912,15 +974,16 @@
       </c>
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="5" t="n"/>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="11" t="n">
         <v>4257</v>
       </c>
-      <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
-      <c r="G17" s="11" t="n">
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="11" t="n">
         <v>1863654</v>
       </c>
-      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -935,11 +998,12 @@
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND LAB 1025 DOKDO CLEANSER_150ml - </t>
+          <t xml:space="preserve">ROUND LAB 1025 DOKDO CLEANSER_150ml </t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
@@ -948,19 +1012,24 @@
       <c r="C19" s="6" t="n">
         <v>599</v>
       </c>
-      <c r="D19" s="6" t="n">
-        <v>779</v>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Cream.Shop 10.8 млн ₽</t>
+        </is>
       </c>
       <c r="E19" s="6" t="n">
         <v>779</v>
       </c>
       <c r="F19" s="6" t="n">
+        <v>779</v>
+      </c>
+      <c r="G19" s="6" t="n">
         <v>291</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="H19" s="6" t="n">
         <v>226689</v>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>держать/растить</t>
         </is>
@@ -969,7 +1038,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB 1025 DOKDO TONER_200ml / Отш</t>
+          <t>ROUND LAB 1025 DOKDO TONER_200ml / О</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
@@ -978,19 +1047,24 @@
       <c r="C20" s="6" t="n">
         <v>81</v>
       </c>
-      <c r="D20" s="6" t="n">
-        <v>0</v>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Cream.Shop 3.0 млн ₽</t>
+        </is>
       </c>
       <c r="E20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6" t="n">
         <v>-419</v>
       </c>
-      <c r="G20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="H20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>минус — резать</t>
         </is>
@@ -999,7 +1073,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB BIRCH JUICE MOISTURIZING CRE</t>
+          <t>ROUND LAB BIRCH JUICE MOISTURIZING C</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
@@ -1008,19 +1082,24 @@
       <c r="C21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D21" s="6" t="n">
-        <v>0</v>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Cream.Shop 5.2 млн ₽</t>
+        </is>
       </c>
       <c r="E21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="6" t="n">
         <v>-543</v>
       </c>
-      <c r="G21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="H21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>минус — резать</t>
         </is>
@@ -1029,7 +1108,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB MUGWORT CALMING CLEANSER_150</t>
+          <t>ROUND LAB MUGWORT CALMING CLEANSER_1</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
@@ -1038,19 +1117,24 @@
       <c r="C22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="6" t="n">
-        <v>120</v>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Cream.Shop 10.8 млн ₽</t>
+        </is>
       </c>
       <c r="E22" s="6" t="n">
         <v>120</v>
       </c>
       <c r="F22" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="G22" s="6" t="n">
         <v>290</v>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="H22" s="6" t="n">
         <v>34800</v>
       </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
@@ -1059,7 +1143,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>ROUND LAB PINE CALMING CICA AMPOULE_30</t>
+          <t>ROUND LAB PINE CALMING CICA AMPOULE_</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
@@ -1068,19 +1152,24 @@
       <c r="C23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="6" t="n">
-        <v>5</v>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Cream.Shop 2.3 млн ₽</t>
+        </is>
       </c>
       <c r="E23" s="6" t="n">
         <v>5</v>
       </c>
       <c r="F23" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="6" t="n">
         <v>290</v>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="H23" s="6" t="n">
         <v>1450</v>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="I23" s="9" t="inlineStr">
         <is>
           <t>ЗАПУСК</t>
         </is>
@@ -1094,15 +1183,16 @@
       </c>
       <c r="B24" s="5" t="n"/>
       <c r="C24" s="5" t="n"/>
-      <c r="D24" s="11" t="n">
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="11" t="n">
         <v>904</v>
       </c>
-      <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
-      <c r="G24" s="11" t="n">
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="11" t="n">
         <v>262939</v>
       </c>
-      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -1117,6 +1207,7 @@
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1130,19 +1221,24 @@
       <c r="C26" s="6" t="n">
         <v>803</v>
       </c>
-      <c r="D26" s="6" t="n">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n">
         <v>1606</v>
       </c>
-      <c r="E26" s="6" t="n">
+      <c r="F26" s="6" t="n">
         <v>402</v>
       </c>
-      <c r="F26" s="6" t="n">
+      <c r="G26" s="6" t="n">
         <v>289</v>
       </c>
-      <c r="G26" s="6" t="n">
+      <c r="H26" s="6" t="n">
         <v>464134</v>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1160,19 +1256,24 @@
       <c r="C27" s="6" t="n">
         <v>1656</v>
       </c>
-      <c r="D27" s="6" t="n">
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n">
         <v>3312</v>
       </c>
-      <c r="E27" s="6" t="n">
+      <c r="F27" s="6" t="n">
         <v>828</v>
       </c>
-      <c r="F27" s="6" t="n">
+      <c r="G27" s="6" t="n">
         <v>198</v>
       </c>
-      <c r="G27" s="6" t="n">
+      <c r="H27" s="6" t="n">
         <v>655776</v>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>держать</t>
         </is>
@@ -1190,19 +1291,24 @@
       <c r="C28" s="6" t="n">
         <v>434</v>
       </c>
-      <c r="D28" s="6" t="n">
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="n">
         <v>868</v>
       </c>
-      <c r="E28" s="6" t="n">
+      <c r="F28" s="6" t="n">
         <v>217</v>
       </c>
-      <c r="F28" s="6" t="n">
+      <c r="G28" s="6" t="n">
         <v>231</v>
       </c>
-      <c r="G28" s="6" t="n">
+      <c r="H28" s="6" t="n">
         <v>200508</v>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1220,19 +1326,24 @@
       <c r="C29" s="6" t="n">
         <v>510</v>
       </c>
-      <c r="D29" s="6" t="n">
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="n">
         <v>1020</v>
       </c>
-      <c r="E29" s="6" t="n">
+      <c r="F29" s="6" t="n">
         <v>255</v>
       </c>
-      <c r="F29" s="6" t="n">
+      <c r="G29" s="6" t="n">
         <v>209</v>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="H29" s="6" t="n">
         <v>213180</v>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>держать</t>
         </is>
@@ -1250,19 +1361,24 @@
       <c r="C30" s="6" t="n">
         <v>296</v>
       </c>
-      <c r="D30" s="6" t="n">
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="n">
         <v>592</v>
       </c>
-      <c r="E30" s="6" t="n">
+      <c r="F30" s="6" t="n">
         <v>148</v>
       </c>
-      <c r="F30" s="6" t="n">
+      <c r="G30" s="6" t="n">
         <v>238</v>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="H30" s="6" t="n">
         <v>140896</v>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1280,19 +1396,24 @@
       <c r="C31" s="6" t="n">
         <v>360</v>
       </c>
-      <c r="D31" s="6" t="n">
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n">
         <v>720</v>
       </c>
-      <c r="E31" s="6" t="n">
+      <c r="F31" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="G31" s="6" t="n">
         <v>224</v>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="H31" s="6" t="n">
         <v>161280</v>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1310,19 +1431,24 @@
       <c r="C32" s="6" t="n">
         <v>310</v>
       </c>
-      <c r="D32" s="6" t="n">
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="n">
         <v>620</v>
       </c>
-      <c r="E32" s="6" t="n">
+      <c r="F32" s="6" t="n">
         <v>155</v>
       </c>
-      <c r="F32" s="6" t="n">
+      <c r="G32" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="G32" s="6" t="n">
+      <c r="H32" s="6" t="n">
         <v>130200</v>
       </c>
-      <c r="H32" s="5" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>держать</t>
         </is>
@@ -1340,19 +1466,24 @@
       <c r="C33" s="6" t="n">
         <v>331</v>
       </c>
-      <c r="D33" s="6" t="n">
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="n">
         <v>662</v>
-      </c>
-      <c r="E33" s="6" t="n">
-        <v>166</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>166</v>
       </c>
       <c r="G33" s="6" t="n">
+        <v>166</v>
+      </c>
+      <c r="H33" s="6" t="n">
         <v>109892</v>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr">
         <is>
           <t>держать</t>
         </is>
@@ -1370,19 +1501,24 @@
       <c r="C34" s="6" t="n">
         <v>209</v>
       </c>
-      <c r="D34" s="6" t="n">
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="n">
         <v>418</v>
       </c>
-      <c r="E34" s="6" t="n">
+      <c r="F34" s="6" t="n">
         <v>104</v>
       </c>
-      <c r="F34" s="6" t="n">
+      <c r="G34" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="G34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="14" t="inlineStr">
+      <c r="H34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="14" t="inlineStr">
         <is>
           <t>не грузить (минус)</t>
         </is>
@@ -1400,19 +1536,24 @@
       <c r="C35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D35" s="6" t="n">
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="E35" s="6" t="n">
+      <c r="F35" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="F35" s="6" t="n">
+      <c r="G35" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="G35" s="6" t="n">
+      <c r="H35" s="6" t="n">
         <v>72000</v>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1430,19 +1571,24 @@
       <c r="C36" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="6" t="n">
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="E36" s="6" t="n">
+      <c r="F36" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="F36" s="6" t="n">
+      <c r="G36" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="G36" s="6" t="n">
+      <c r="H36" s="6" t="n">
         <v>72000</v>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1460,19 +1606,24 @@
       <c r="C37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D37" s="6" t="n">
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="E37" s="6" t="n">
+      <c r="F37" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="F37" s="6" t="n">
+      <c r="G37" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="G37" s="6" t="n">
+      <c r="H37" s="6" t="n">
         <v>72000</v>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1490,19 +1641,24 @@
       <c r="C38" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="6" t="n">
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="E38" s="6" t="n">
+      <c r="F38" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="F38" s="6" t="n">
+      <c r="G38" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="G38" s="6" t="n">
+      <c r="H38" s="6" t="n">
         <v>72000</v>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="I38" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1520,19 +1676,24 @@
       <c r="C39" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D39" s="6" t="n">
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="E39" s="6" t="n">
+      <c r="F39" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="F39" s="6" t="n">
+      <c r="G39" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="H39" s="6" t="n">
         <v>72000</v>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1550,19 +1711,24 @@
       <c r="C40" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D40" s="6" t="n">
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>— (сезонка)</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="E40" s="6" t="n">
+      <c r="F40" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="F40" s="6" t="n">
+      <c r="G40" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="H40" s="6" t="n">
         <v>37800</v>
       </c>
-      <c r="H40" s="5" t="inlineStr">
+      <c r="I40" s="5" t="inlineStr">
         <is>
           <t>разгонять</t>
         </is>
@@ -1576,68 +1742,61 @@
       </c>
       <c r="B41" s="5" t="n"/>
       <c r="C41" s="5" t="n"/>
-      <c r="D41" s="11" t="n">
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="11" t="n">
         <v>12028</v>
       </c>
-      <c r="E41" s="11" t="n">
+      <c r="F41" s="11" t="n">
         <v>3007</v>
       </c>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="11" t="n">
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="11" t="n">
         <v>2473666</v>
       </c>
-      <c r="H41" s="5" t="n"/>
+      <c r="I41" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>ИТОГО ОКТЯБРЬ (косметика + ramp Санты): 2 745 010 ₽  8 168 шт</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="15" t="inlineStr">
-        <is>
-          <t>СПРАВОЧНО — полный Q4: 4 600 259 ₽</t>
+          <t>ИТОГО ОКТЯБРЬ: 2 745 010 ₽  8 168 шт  ·  полный Q4: 4 600 259 ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>Celimax: конкурент LIFECOSM — его продажи в шт/мес по тому же товару (из отчёта Ozon по его товарам).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>Petitfee убран из плана (на Озоне почти не продавался).</t>
+          <t>Round Lab: конкурент Cream.Shop — его продажи Round Lab по категории в ₽/мес (данные только по категориям; Cream.Shop держит ~73% рынка Round Lab-умывания).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>ВАЖНО: остаток Санты (43 тыс.) общий с WB — прогноз на Озон не складывать с WB-планом.</t>
+          <t>Petitfee убран. Остаток Санты общий с WB — не складывать с WB-планом. На FBO грузим только прогноз.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>На FBO грузим только прогноз Санты, не весь остаток (72% не продастся за сезон).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="16" t="inlineStr">
-        <is>
-          <t>Итоги — цель при исполнении (реклама ≤15% ДРР, запуск показов Retinal, раскладка по кластерам). Реалистичный пол по косметике ~0,9–1,1 млн.</t>
+          <t>Прибыль — цель при исполнении; реалистичный пол по косметике ~0,9–1,1 млн/мес.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A46:H46"/>
+  <mergeCells count="5">
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A48:I48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Santa block: use current stock only (exclude in-transit container)
Per owner: plan Santa on current 30852 units only; drop container-only
models (2,7,8,15). Season forecast ~10330, rest not shipped to FBO.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
+++ b/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Конкурент: Celimax → LIFECOSM (шт/мес, по товару); Round Lab → Cream.Shop (₽/мес по категории, ~73% рынка Round Lab).</t>
+          <t>Санта — ТОЛЬКО текущий остаток (контейнер в пути не учтён). Конкурент: Celimax→LIFECOSM (шт), Round Lab→Cream.Shop (₽ по кат.).</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>ДЕДЫ МОРОЗЫ · сезон Q4 (Озон)</t>
+          <t>ДЕДЫ МОРОЗЫ · сезон Q4 (Озон, текущий остаток)</t>
         </is>
       </c>
       <c r="B25" s="13" t="n"/>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>10885</v>
+        <v>4987</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>803</v>
@@ -1286,7 +1286,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>7463</v>
+        <v>5819</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>434</v>
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>2374</v>
+        <v>1444</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>331</v>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>1497</v>
+        <v>717</v>
       </c>
       <c r="C35" s="6" t="n">
         <v>0</v>
@@ -1542,16 +1542,16 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G35" s="6" t="n">
         <v>180</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>72000</v>
+        <v>54000</v>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>722</v>
+        <v>212</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>400</v>
+        <v>212</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="G36" s="6" t="n">
         <v>180</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>72000</v>
+        <v>38160</v>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
@@ -1595,196 +1595,56 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>№2 (нов)</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="n">
-        <v>990</v>
-      </c>
-      <c r="C37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>— (сезонка)</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="H37" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>№7 (нов)</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n">
-        <v>930</v>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>— (сезонка)</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="F38" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="G38" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="H38" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Итого Деды Морозы (сезон)</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="11" t="n">
+        <v>10330</v>
+      </c>
+      <c r="F37" s="11" t="n">
+        <v>2583</v>
+      </c>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="11" t="n">
+        <v>2168026</v>
+      </c>
+      <c r="I37" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>№8 (нов)</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="n">
-        <v>576</v>
-      </c>
-      <c r="C39" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>— (сезонка)</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="F39" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="G39" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="H39" s="6" t="n">
-        <v>72000</v>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>№15 (нов)</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="C40" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>— (сезонка)</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="F40" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="G40" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="H40" s="6" t="n">
-        <v>37800</v>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>разгонять</t>
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>ИТОГО ОКТЯБРЬ: 2 668 600 ₽  7 744 шт  ·  полный Q4: 4 294 619 ₽</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Итого Деды Морозы (сезон)</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="11" t="n">
-        <v>12028</v>
-      </c>
-      <c r="F41" s="11" t="n">
-        <v>3007</v>
-      </c>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="11" t="n">
-        <v>2473666</v>
-      </c>
-      <c r="I41" s="5" t="n"/>
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Санта: учтён ТОЛЬКО текущий остаток 30 852 шт (контейнер в пути пока не считаем). Прогноз сезона ~10 330 шт — остальное не грузить на FBO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>Celimax: конкурент LIFECOSM (шт/мес по товару). Round Lab: Cream.Shop (₽/мес по категории, ~73% рынка Round Lab-умывания).</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="15" t="inlineStr">
-        <is>
-          <t>ИТОГО ОКТЯБРЬ: 2 745 010 ₽  8 168 шт  ·  полный Q4: 4 600 259 ₽</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>Celimax: конкурент LIFECOSM — его продажи в шт/мес по тому же товару (из отчёта Ozon по его товарам).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="16" t="inlineStr">
-        <is>
-          <t>Round Lab: конкурент Cream.Shop — его продажи Round Lab по категории в ₽/мес (данные только по категориям; Cream.Shop держит ~73% рынка Round Lab-умывания).</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>Petitfee убран. Остаток Санты общий с WB — не складывать с WB-планом. На FBO грузим только прогноз.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>Petitfee убран. Остаток Санты общий с WB — не складывать с WB-планом.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>Прибыль — цель при исполнении; реалистичный пол по косметике ~0,9–1,1 млн/мес.</t>
         </is>
@@ -1793,10 +1653,10 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A43:I43"/>
-    <mergeCell ref="A47:I47"/>
-    <mergeCell ref="A46:I46"/>
-    <mergeCell ref="A45:I45"/>
-    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A39:I39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Show Cream.Shop (Round Lab) benchmark in units not RUB
Cream.Shop Round Lab category units/mo: cleanser 9560, toner 2062,
cream 3231, serum 1522. Matches LIFECOSM units column for Celimax.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
+++ b/outputs/ozon_sales_plan/ozon_sales_plan_october_full_2026.xlsx
@@ -491,13 +491,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -508,14 +508,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OZON — план: косметика (Celimax, Round Lab) + Деды Морозы, с конкурентами</t>
+          <t>OZON — план: косметика (Celimax, Round Lab) + Деды Морозы, с конкурентами (в шт)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Санта — ТОЛЬКО текущий остаток (контейнер в пути не учтён). Конкурент: Celimax→LIFECOSM (шт), Round Lab→Cream.Shop (₽ по кат.).</t>
+          <t>Санта — только текущий остаток. Конкурент (шт/мес): Celimax→LIFECOSM (по товару), Round Lab→Cream.Shop (по категории).</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Конкурент (прод.)</t>
+          <t>Конкурент, шт/мес</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 4354 шт</t>
+          <t>LIFECOSM 4354</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
@@ -630,7 +630,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 4295 шт</t>
+          <t>LIFECOSM 4295</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
@@ -665,7 +665,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 1423 шт</t>
+          <t>LIFECOSM 1423</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
@@ -700,7 +700,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 4560 шт</t>
+          <t>LIFECOSM 4560</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
@@ -770,7 +770,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 850 шт</t>
+          <t>LIFECOSM 850</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
@@ -805,7 +805,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 850 шт</t>
+          <t>LIFECOSM 850</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 928 шт</t>
+          <t>LIFECOSM 928</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
@@ -875,7 +875,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 1080 шт</t>
+          <t>LIFECOSM 1080</t>
         </is>
       </c>
       <c r="E14" s="6" t="n">
@@ -910,7 +910,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 584 шт</t>
+          <t>LIFECOSM 584</t>
         </is>
       </c>
       <c r="E15" s="6" t="n">
@@ -945,7 +945,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>LIFECOSM 1399 шт</t>
+          <t>LIFECOSM 1399</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Cream.Shop 10.8 млн ₽</t>
+          <t>Cream.Shop 9560*</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Cream.Shop 3.0 млн ₽</t>
+          <t>Cream.Shop 2062*</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Cream.Shop 5.2 млн ₽</t>
+          <t>Cream.Shop 3231*</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Cream.Shop 10.8 млн ₽</t>
+          <t>Cream.Shop 9560*</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Cream.Shop 2.3 млн ₽</t>
+          <t>Cream.Shop 1522*</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
@@ -1625,37 +1625,29 @@
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>Санта: учтён ТОЛЬКО текущий остаток 30 852 шт (контейнер в пути пока не считаем). Прогноз сезона ~10 330 шт — остальное не грузить на FBO.</t>
+          <t>* Cream.Shop — шт/мес по КАТЕГОРИИ Round Lab (умывание 9 560, тонер 2 062, крем 3 231, сыворотка 1 522), т.к. по-товарной разбивки конкурента нет. LIFECOSM — по товару.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>Celimax: конкурент LIFECOSM (шт/мес по товару). Round Lab: Cream.Shop (₽/мес по категории, ~73% рынка Round Lab-умывания).</t>
+          <t>Санта — только текущий остаток 30 852 шт (контейнер не учтён). На FBO грузим только прогноз, остальное не везти.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>Petitfee убран. Остаток Санты общий с WB — не складывать с WB-планом.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>Прибыль — цель при исполнении; реалистичный пол по косметике ~0,9–1,1 млн/мес.</t>
+          <t>Petitfee убран. Остаток Санты общий с WB. Прибыль — цель; пол по косметике ~0,9–1,1 млн/мес.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
+    <mergeCell ref="A42:I42"/>
     <mergeCell ref="A43:I43"/>
     <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A42:I42"/>
-    <mergeCell ref="A44:I44"/>
     <mergeCell ref="A39:I39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>